<commit_message>
Fix mm/inch section width data, format tire spec charts to 1 decimal
Section Width was entered in mm for three tires (Neo Fuel D3, Neo Fuel
G3, Neo Allroads S) instead of inches; corrected in the wireframe and
regenerated the tire catalog. Also format Section Width, Overall
Diameter, and Tread Depth (32nds) to a consistent single decimal place
on the product page spec table, matching the Tire Finder page.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Aeolus-Wireframe-06.xlsx
+++ b/Aeolus-Wireframe-06.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cld\Aeolus-Tire\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ECC380A-6CB4-4314-A311-14226883891B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5851CE78-194A-4F28-BEAE-842112E97F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30720" yWindow="552" windowWidth="23040" windowHeight="13740" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18936" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Support" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4462" uniqueCount="664">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4459" uniqueCount="661">
   <si>
     <t>Tire Name</t>
   </si>
@@ -2024,15 +2024,6 @@
     <t>The new dual-layer tread structure uses a medium- and long-distance compound formulation to balance mileage and heat dissipation, maintaining durability and performance even under heavy-duty operations.</t>
   </si>
   <si>
-    <t>ai rec' 12.2</t>
-  </si>
-  <si>
-    <t>ai rec' 11.6</t>
-  </si>
-  <si>
-    <t>ai rec' 11.7</t>
-  </si>
-  <si>
     <t>Designed for use on “Last mile” Delivery Vehicle</t>
   </si>
   <si>
@@ -2240,7 +2231,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2310,12 +2301,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2403,7 +2388,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="159">
+  <cellXfs count="157">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -2840,12 +2825,8 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -20357,9 +20338,7 @@
       <c r="Y105" s="52"/>
     </row>
     <row r="106" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A106" s="158" t="s">
-        <v>659</v>
-      </c>
+      <c r="A106" s="52"/>
       <c r="B106" s="69"/>
       <c r="C106" s="64"/>
       <c r="E106" s="35" t="s">
@@ -20371,8 +20350,8 @@
       <c r="G106" s="36">
         <v>9</v>
       </c>
-      <c r="H106" s="157">
-        <v>297</v>
+      <c r="H106" s="156">
+        <v>11.7</v>
       </c>
       <c r="I106" s="37">
         <v>40.4</v>
@@ -24836,9 +24815,7 @@
       <c r="Y243" s="52"/>
     </row>
     <row r="244" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A244" s="158" t="s">
-        <v>658</v>
-      </c>
+      <c r="A244" s="52"/>
       <c r="B244" s="69"/>
       <c r="C244" s="64"/>
       <c r="E244" s="35" t="s">
@@ -24850,8 +24827,8 @@
       <c r="G244" s="36">
         <v>9</v>
       </c>
-      <c r="H244" s="157">
-        <v>296</v>
+      <c r="H244" s="156">
+        <v>11.7</v>
       </c>
       <c r="I244" s="37">
         <v>39.9</v>
@@ -26018,9 +25995,7 @@
       <c r="Y278" s="52"/>
     </row>
     <row r="279" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A279" s="158" t="s">
-        <v>657</v>
-      </c>
+      <c r="A279" s="52"/>
       <c r="B279" s="69"/>
       <c r="C279" s="64"/>
       <c r="E279" s="35" t="s">
@@ -26032,8 +26007,8 @@
       <c r="G279" s="36">
         <v>9</v>
       </c>
-      <c r="H279" s="157">
-        <v>309</v>
+      <c r="H279" s="156">
+        <v>11.7</v>
       </c>
       <c r="I279" s="37">
         <v>41.7</v>
@@ -32685,7 +32660,7 @@
       </c>
       <c r="B463" s="70"/>
       <c r="C463" s="73"/>
-      <c r="D463" s="156" t="s">
+      <c r="D463" t="s">
         <v>655</v>
       </c>
       <c r="E463" s="52"/>
@@ -32805,7 +32780,7 @@
       </c>
       <c r="B467" s="70"/>
       <c r="C467" s="73"/>
-      <c r="D467" s="156" t="s">
+      <c r="D467" t="s">
         <v>656</v>
       </c>
       <c r="E467" s="52"/>
@@ -49883,7 +49858,7 @@
       <c r="B959" s="70"/>
       <c r="C959" s="73"/>
       <c r="D959" s="52" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="E959" s="52"/>
       <c r="F959" s="52"/>
@@ -54101,7 +54076,7 @@
       </c>
       <c r="B1083" s="70"/>
       <c r="C1083" s="87" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="D1083" s="52"/>
       <c r="E1083" s="52"/>
@@ -54280,7 +54255,7 @@
       <c r="B1089" s="70"/>
       <c r="C1089" s="73"/>
       <c r="D1089" s="78" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="E1089" s="52"/>
       <c r="F1089" s="52"/>
@@ -70525,7 +70500,7 @@
       </c>
       <c r="B1558" s="70"/>
       <c r="C1558" s="87" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="D1558" s="52"/>
       <c r="E1558" s="52"/>

</xml_diff>

<commit_message>
Feature real tires in homepage product grid with photos and links
Replace the concept-stage "Best Sellers" grid (same tire duplicated
three times, fabricated spec labels) with Neo Fuel D3, Neo Construct G,
and ADW82 sourced live from CATALOG_TIRES. Cards now show the tire's
real photo cropped to the site's standard thumbnail framing, link to
the product page, and dim to 70% opacity until hovered.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Aeolus-Wireframe-06.xlsx
+++ b/Aeolus-Wireframe-06.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cld\Aeolus-Tire\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ED13743E-E722-4932-927F-5743CAFC6D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27D5249F-8DF4-4BEF-BD44-A6471EC69A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18936" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="23256" windowHeight="14616" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Support" sheetId="1" r:id="rId1"/>
@@ -3945,7 +3945,7 @@
     <col min="20" max="20" width="9.44140625" style="12" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="5.6640625" style="14" customWidth="1"/>
     <col min="22" max="22" width="5.21875" style="14" customWidth="1"/>
-    <col min="23" max="23" width="6.44140625" style="14" customWidth="1"/>
+    <col min="23" max="23" width="6.44140625" style="14" hidden="1" customWidth="1"/>
     <col min="24" max="24" width="11.6640625" style="5" hidden="1" customWidth="1"/>
     <col min="26" max="26" width="2.21875" customWidth="1"/>
     <col min="31" max="31" width="20.77734375" customWidth="1"/>

</xml_diff>